<commit_message>
Improve dashboard header branding
</commit_message>
<xml_diff>
--- a/downloads/offer-evidence.xlsx
+++ b/downloads/offer-evidence.xlsx
@@ -1856,11 +1856,7 @@
           <t>https://front.alforaij.com/Listing/Detail/303</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c1d220d219ce4ccd894d4913b311728b.png</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2126,11 +2122,7 @@
           <t>https://front.alforaij.com/Listing/Detail/301</t>
         </is>
       </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/225dfeaa91bb41018e81acd75d76bc7c.jpeg</t>
-        </is>
-      </c>
+      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2478,7 +2470,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -2496,11 +2488,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4167,11 +4155,7 @@
           <t>https://front.alforaij.com/Listing/Detail/276</t>
         </is>
       </c>
-      <c r="R33" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/2772f7b538bc480d8812dc4d909d8621.png</t>
-        </is>
-      </c>
+      <c r="R33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -24626,613 +24610,609 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q174" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R174" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q175" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q176" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q177" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R177" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q178" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R178" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q179" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q180" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R180" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R181" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R182" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q183" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R183" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q184" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q185" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R185" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q186" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R186" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q187" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R187" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q188" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R188" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q189" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R189" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R191" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q192" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R192" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q193" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R194" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R195" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q196" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R196" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q197" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q198" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q199" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R199" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q200" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q201" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R201" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q202" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R202" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q203" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q204" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q205" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q206" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q207" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R207" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R208" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q210" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q211" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q212" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q213" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q214" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R214" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q215" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q216" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R216" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q217" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q218" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R218" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q219" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R219" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q220" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R220" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R221" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q222" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q223" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q224" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R224" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q225" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q226" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R226" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q227" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q228" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q229" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q230" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q231" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q232" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q233" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q234" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q235" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R235" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q236" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q237" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q239" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R239" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q240" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R240" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q241" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R241" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q242" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R242" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q243" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R243" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q244" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q245" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R245" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q246" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R246" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q247" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R247" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q248" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R248" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q249" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R249" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q250" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R250" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q251" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R251" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q252" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R252" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q253" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R253" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q254" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R254" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q255" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q256" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R256" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q257" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q258" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R258" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q259" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R259" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q260" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R260" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q261" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R261" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q262" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R262" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q263" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R263" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q264" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q265" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R265" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q266" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R266" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q267" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R267" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q268" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q269" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q270" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q271" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R271" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q272" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q273" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R273" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q274" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R274" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q275" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R275" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q276" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R276" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q174" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R174" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q175" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q176" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q177" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R177" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q178" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R178" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q179" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q180" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R180" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R181" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R182" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q183" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R183" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q184" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q185" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R185" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q186" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R186" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q187" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R187" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q188" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R188" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q189" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R189" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R191" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q192" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R192" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q193" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R194" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R195" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q196" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R196" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q197" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q198" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q199" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R199" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q200" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q201" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R201" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q202" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R202" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q203" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q204" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q205" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q206" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q207" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R207" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R208" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q210" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q211" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q212" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q213" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q214" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R214" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q215" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q216" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R216" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q217" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q218" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R218" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q219" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R219" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q220" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R220" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R221" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q222" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q223" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q224" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R224" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q225" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q226" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R226" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q227" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q228" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q229" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q230" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q231" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q232" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q233" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q234" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q235" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R235" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q236" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q237" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q239" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R239" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q240" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R240" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q241" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R241" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q242" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R242" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q243" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R243" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q244" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q245" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R245" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q246" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R246" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q247" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R247" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q248" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R248" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q249" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R249" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q250" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R250" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q251" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R251" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q252" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R252" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q253" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R253" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q254" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R254" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q255" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q256" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R256" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q257" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q258" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R258" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q259" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R259" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q260" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R260" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q261" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R261" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q262" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R262" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q263" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R263" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q264" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q265" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R265" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q266" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R266" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q267" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R267" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q268" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q269" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q270" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q271" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R271" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q272" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q273" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R273" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q274" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R274" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q275" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R275" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q276" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R276" r:id="rId619"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId624"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId620"/>
   </tableParts>
 </worksheet>
 </file>
@@ -25880,11 +25860,7 @@
           <t>https://front.alforaij.com/Listing/Detail/303</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c1d220d219ce4ccd894d4913b311728b.png</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -26056,11 +26032,7 @@
           <t>https://front.alforaij.com/Listing/Detail/301</t>
         </is>
       </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/225dfeaa91bb41018e81acd75d76bc7c.jpeg</t>
-        </is>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -26122,7 +26094,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -26140,11 +26112,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -26832,11 +26800,7 @@
           <t>https://front.alforaij.com/Listing/Detail/276</t>
         </is>
       </c>
-      <c r="R18" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/2772f7b538bc480d8812dc4d909d8621.png</t>
-        </is>
-      </c>
+      <c r="R18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -41719,414 +41683,410 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q174" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q175" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q176" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q177" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q178" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R178" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q179" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R179" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q180" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R180" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R181" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R182" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q183" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R183" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q184" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q185" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R185" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q186" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R186" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q187" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R187" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q188" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q189" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R190" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q192" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R192" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q193" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R193" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R194" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R195" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q174" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q175" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q176" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q177" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q178" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R178" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q179" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R179" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q180" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R180" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R181" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R182" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q183" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R183" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q184" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q185" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R185" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q186" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R186" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q187" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R187" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q188" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q189" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R190" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q192" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R192" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q193" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R193" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R194" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R195" r:id="rId417"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId422"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId418"/>
   </tableParts>
 </worksheet>
 </file>
@@ -45610,11 +45570,7 @@
           <t>https://front.alforaij.com/Listing/Detail/303</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c1d220d219ce4ccd894d4913b311728b.png</t>
-        </is>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -45786,11 +45742,7 @@
           <t>https://front.alforaij.com/Listing/Detail/301</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/225dfeaa91bb41018e81acd75d76bc7c.jpeg</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -56296,293 +56248,291 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId295"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId298"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId296"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Optimize dashboard initial load
</commit_message>
<xml_diff>
--- a/downloads/offer-evidence.xlsx
+++ b/downloads/offer-evidence.xlsx
@@ -1392,11 +1392,7 @@
           <t>https://front.alforaij.com/Listing/Detail/303</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c1d220d219ce4ccd894d4913b311728b.png</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1480,11 +1476,7 @@
           <t>https://front.alforaij.com/Listing/Detail/302</t>
         </is>
       </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/f77fdc541be74b11b6f2d504c2c4ab56.jpeg</t>
-        </is>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2816,11 +2808,7 @@
           <t>https://front.alforaij.com/Listing/Detail/287</t>
         </is>
       </c>
-      <c r="R23" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/52aee6671a62401993af77f7512817b4.png</t>
-        </is>
-      </c>
+      <c r="R23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3357,11 +3345,7 @@
           <t>https://front.alforaij.com/Listing/Detail/280</t>
         </is>
       </c>
-      <c r="R29" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c28ac06bd5f149208ec5b361dbd04434.png</t>
-        </is>
-      </c>
+      <c r="R29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3513,7 +3497,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -3531,11 +3515,7 @@
           <t>https://front.alforaij.com/Listing/Detail/278</t>
         </is>
       </c>
-      <c r="R31" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/7250c1cdf2fd4b79935f9d400a1ff2b9.png</t>
-        </is>
-      </c>
+      <c r="R31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8525,7 +8505,14 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>🏢 للبيع برج استثماري فاخر في منطقة الفروانية
+📍 الموقع: موقع حيوي واستراتيجي جداً (بجانب فندق كراون بلازا)
+📐 مساحة الأرض: 750 متر مربع
+🏗️ التصنيف:</t>
+        </is>
+      </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -8556,7 +8543,11 @@
           <t>https://front.alforaij.com/Listing/Detail/188</t>
         </is>
       </c>
-      <c r="R86" s="2" t="inlineStr"/>
+      <c r="R86" s="3" t="inlineStr">
+        <is>
+          <t>https://search.alforaij.com/uploads/internallistings/f11fa5ea5cb84d658a6e1646a11bb275.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -16358,502 +16349,498 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId508"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId513"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId509"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17501,11 +17488,7 @@
           <t>https://front.alforaij.com/Listing/Detail/303</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c1d220d219ce4ccd894d4913b311728b.png</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -17589,11 +17572,7 @@
           <t>https://front.alforaij.com/Listing/Detail/302</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/f77fdc541be74b11b6f2d504c2c4ab56.jpeg</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -17847,11 +17826,7 @@
           <t>https://front.alforaij.com/Listing/Detail/287</t>
         </is>
       </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/52aee6671a62401993af77f7512817b4.png</t>
-        </is>
-      </c>
+      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -18107,11 +18082,7 @@
           <t>https://front.alforaij.com/Listing/Detail/280</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c28ac06bd5f149208ec5b361dbd04434.png</t>
-        </is>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -18263,7 +18234,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
@@ -18281,11 +18252,7 @@
           <t>https://front.alforaij.com/Listing/Detail/278</t>
         </is>
       </c>
-      <c r="R16" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/7250c1cdf2fd4b79935f9d400a1ff2b9.png</t>
-        </is>
-      </c>
+      <c r="R16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -22043,7 +22010,14 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>🏢 للبيع برج استثماري فاخر في منطقة الفروانية
+📍 الموقع: موقع حيوي واستراتيجي جداً (بجانب فندق كراون بلازا)
+📐 مساحة الأرض: 750 متر مربع
+🏗️ التصنيف:</t>
+        </is>
+      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -22074,7 +22048,11 @@
           <t>https://front.alforaij.com/Listing/Detail/188</t>
         </is>
       </c>
-      <c r="R58" s="2" t="inlineStr"/>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>https://search.alforaij.com/uploads/internallistings/f11fa5ea5cb84d658a6e1646a11bb275.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -27047,325 +27025,321 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId328"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId333"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId329"/>
   </tableParts>
 </worksheet>
 </file>
@@ -30780,11 +30754,7 @@
           <t>https://front.alforaij.com/Listing/Detail/303</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c1d220d219ce4ccd894d4913b311728b.png</t>
-        </is>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -30868,11 +30838,7 @@
           <t>https://front.alforaij.com/Listing/Detail/302</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/f77fdc541be74b11b6f2d504c2c4ab56.jpeg</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -31042,11 +31008,7 @@
           <t>https://front.alforaij.com/Listing/Detail/287</t>
         </is>
       </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/52aee6671a62401993af77f7512817b4.png</t>
-        </is>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -31286,7 +31248,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
@@ -31304,11 +31266,7 @@
           <t>https://front.alforaij.com/Listing/Detail/278</t>
         </is>
       </c>
-      <c r="R12" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/7250c1cdf2fd4b79935f9d400a1ff2b9.png</t>
-        </is>
-      </c>
+      <c r="R12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -37761,242 +37719,238 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId242"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId247"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId243"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve mobile layout and external images
</commit_message>
<xml_diff>
--- a/downloads/offer-evidence.xlsx
+++ b/downloads/offer-evidence.xlsx
@@ -848,7 +848,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -866,11 +866,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1091,15 +1087,7 @@
           <t>مباشر</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع في مدينة صباح الأحمد السكنية
-📐 المساحة: 400 متر مربع
-📞 للاستفسار والتواصل:
-📱 55559950 | 📱 41060118
-🌐 alforaij.com</t>
-        </is>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -1130,11 +1118,7 @@
           <t>https://front.alforaij.com/Listing/Detail/306</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c5c2770212744270b644516a73ff9273.jpeg</t>
-        </is>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1304,11 +1288,7 @@
           <t>https://front.alforaij.com/Listing/Detail/304</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/076f2bc4192840a5af5ab3ff657177d6.jpeg</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2014,7 +1994,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -2032,11 +2012,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3846,14 +3822,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -3884,11 +3853,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -16351,521 +16316,516 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId508"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId514"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId509"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17055,7 +17015,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -17073,11 +17033,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -17212,15 +17168,7 @@
           <t>مباشر</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع في مدينة صباح الأحمد السكنية
-📐 المساحة: 400 متر مربع
-📞 للاستفسار والتواصل:
-📱 55559950 | 📱 41060118
-🌐 alforaij.com</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -17251,11 +17199,7 @@
           <t>https://front.alforaij.com/Listing/Detail/306</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c5c2770212744270b644516a73ff9273.jpeg</t>
-        </is>
-      </c>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -17425,11 +17369,7 @@
           <t>https://front.alforaij.com/Listing/Detail/304</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/076f2bc4192840a5af5ab3ff657177d6.jpeg</t>
-        </is>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -17755,7 +17695,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -17773,11 +17713,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -18516,14 +18452,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -18554,11 +18483,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R19" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -27055,341 +26980,336 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId328"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId334"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId329"/>
   </tableParts>
 </worksheet>
 </file>
@@ -30434,7 +30354,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -30452,11 +30372,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -30591,15 +30507,7 @@
           <t>مباشر</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع في مدينة صباح الأحمد السكنية
-📐 المساحة: 400 متر مربع
-📞 للاستفسار والتواصل:
-📱 55559950 | 📱 41060118
-🌐 alforaij.com</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -30630,11 +30538,7 @@
           <t>https://front.alforaij.com/Listing/Detail/306</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c5c2770212744270b644516a73ff9273.jpeg</t>
-        </is>
-      </c>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -31465,14 +31369,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -31503,11 +31400,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -37773,254 +37666,251 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId243"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId247"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId244"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Sync metric cards with governorate table
</commit_message>
<xml_diff>
--- a/downloads/offer-evidence.xlsx
+++ b/downloads/offer-evidence.xlsx
@@ -848,7 +848,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -866,11 +866,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1662,11 +1658,7 @@
           <t>https://front.alforaij.com/Listing/Detail/301</t>
         </is>
       </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/225dfeaa91bb41018e81acd75d76bc7c.jpeg</t>
-        </is>
-      </c>
+      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2014,7 +2006,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -2032,11 +2024,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3846,14 +3834,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -3884,11 +3865,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -16351,521 +16328,517 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId509"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId514"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId510"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17055,7 +17028,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -17073,11 +17046,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -17689,11 +17658,7 @@
           <t>https://front.alforaij.com/Listing/Detail/301</t>
         </is>
       </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/225dfeaa91bb41018e81acd75d76bc7c.jpeg</t>
-        </is>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -17755,7 +17720,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -17773,11 +17738,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -18516,14 +18477,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -18554,11 +18508,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R19" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -27055,341 +27005,337 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId329"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId334"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId330"/>
   </tableParts>
 </worksheet>
 </file>
@@ -30434,7 +30380,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -30452,11 +30398,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -30980,11 +30922,7 @@
           <t>https://front.alforaij.com/Listing/Detail/301</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/225dfeaa91bb41018e81acd75d76bc7c.jpeg</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -31465,14 +31403,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -31503,11 +31434,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -37773,254 +37700,251 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId243"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId247"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId244"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Sync governorate table clicks with metric cards
</commit_message>
<xml_diff>
--- a/downloads/offer-evidence.xlsx
+++ b/downloads/offer-evidence.xlsx
@@ -848,7 +848,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -866,11 +866,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1091,15 +1087,7 @@
           <t>مباشر</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع في مدينة صباح الأحمد السكنية
-📐 المساحة: 400 متر مربع
-📞 للاستفسار والتواصل:
-📱 55559950 | 📱 41060118
-🌐 alforaij.com</t>
-        </is>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -1130,11 +1118,7 @@
           <t>https://front.alforaij.com/Listing/Detail/306</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c5c2770212744270b644516a73ff9273.jpeg</t>
-        </is>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1216,11 +1200,7 @@
           <t>https://front.alforaij.com/Listing/Detail/305</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/0a733896943b4a1ba99a097d7716d7bb.jpeg</t>
-        </is>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1480,11 +1460,7 @@
           <t>https://front.alforaij.com/Listing/Detail/302</t>
         </is>
       </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/f77fdc541be74b11b6f2d504c2c4ab56.jpeg</t>
-        </is>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2014,7 +1990,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -2032,11 +2008,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3357,11 +3329,7 @@
           <t>https://front.alforaij.com/Listing/Detail/280</t>
         </is>
       </c>
-      <c r="R29" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c28ac06bd5f149208ec5b361dbd04434.png</t>
-        </is>
-      </c>
+      <c r="R29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3846,14 +3814,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -3884,11 +3845,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -16351,521 +16308,514 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId506"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId514"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId507"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17055,7 +17005,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -17073,11 +17023,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -17212,15 +17158,7 @@
           <t>مباشر</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع في مدينة صباح الأحمد السكنية
-📐 المساحة: 400 متر مربع
-📞 للاستفسار والتواصل:
-📱 55559950 | 📱 41060118
-🌐 alforaij.com</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -17251,11 +17189,7 @@
           <t>https://front.alforaij.com/Listing/Detail/306</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c5c2770212744270b644516a73ff9273.jpeg</t>
-        </is>
-      </c>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -17337,11 +17271,7 @@
           <t>https://front.alforaij.com/Listing/Detail/305</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/0a733896943b4a1ba99a097d7716d7bb.jpeg</t>
-        </is>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -17601,11 +17531,7 @@
           <t>https://front.alforaij.com/Listing/Detail/302</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/f77fdc541be74b11b6f2d504c2c4ab56.jpeg</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -17755,7 +17681,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -17773,11 +17699,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -18119,11 +18041,7 @@
           <t>https://front.alforaij.com/Listing/Detail/280</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c28ac06bd5f149208ec5b361dbd04434.png</t>
-        </is>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -18516,14 +18434,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -18554,11 +18465,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R19" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -27055,341 +26962,334 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId326"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId334"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId327"/>
   </tableParts>
 </worksheet>
 </file>
@@ -30434,7 +30334,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>نعم</t>
+          <t>لا</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -30452,11 +30352,7 @@
           <t>https://front.alforaij.com/Listing/Detail/309</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/560deeb22a734fb683f1805dafb2d3c7.png</t>
-        </is>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -30591,15 +30487,7 @@
           <t>مباشر</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع في مدينة صباح الأحمد السكنية
-📐 المساحة: 400 متر مربع
-📞 للاستفسار والتواصل:
-📱 55559950 | 📱 41060118
-🌐 alforaij.com</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>ساحة</t>
@@ -30630,11 +30518,7 @@
           <t>https://front.alforaij.com/Listing/Detail/306</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/c5c2770212744270b644516a73ff9273.jpeg</t>
-        </is>
-      </c>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -30716,11 +30600,7 @@
           <t>https://front.alforaij.com/Listing/Detail/305</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/0a733896943b4a1ba99a097d7716d7bb.jpeg</t>
-        </is>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -30892,11 +30772,7 @@
           <t>https://front.alforaij.com/Listing/Detail/302</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/f77fdc541be74b11b6f2d504c2c4ab56.jpeg</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -31465,14 +31341,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>📍 للبيع فيلا في منطقة الشهداء (قطعة 2)
-📐 المساحة: 375 متر مربع (بنيان 2017)
-🗺️ الموقع: بطن وظهر (ارتداد مميز أكثر من 100 متر)
-🌐 رابط الموقع (كويت</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>بطن وظهر، ارتداد، ساحة</t>
@@ -31503,11 +31372,7 @@
           <t>https://front.alforaij.com/Listing/Detail/274</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/d7ee2603bec94fc7aac4c12e99d09385.png</t>
-        </is>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -37773,254 +37638,249 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId241"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId247"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId242"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Optimize dashboard data and mobile experience
</commit_message>
<xml_diff>
--- a/downloads/offer-evidence.xlsx
+++ b/downloads/offer-evidence.xlsx
@@ -2120,11 +2120,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R16" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3531,11 +3527,7 @@
           <t>https://front.alforaij.com/Listing/Detail/279</t>
         </is>
       </c>
-      <c r="R31" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/8fd44f6b937742e4b64fccbaf940d5c3.png</t>
-        </is>
-      </c>
+      <c r="R31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -16481,482 +16473,480 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R173" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q113" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R113" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q114" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R114" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q115" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R115" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q116" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R116" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q117" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R117" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q118" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R118" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q119" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R119" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q120" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R120" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R121" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R122" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R123" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R124" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R125" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R126" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R127" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R128" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R129" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R130" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R131" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R132" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R133" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R134" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R135" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R136" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R137" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R138" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R139" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R140" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R141" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R142" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R143" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R144" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R145" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R146" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R147" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R148" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R149" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R150" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R151" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R152" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R153" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R154" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R155" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R156" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R157" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R158" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R159" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R160" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R161" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R162" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R163" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R164" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R165" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R166" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R167" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R168" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R169" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R170" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R171" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R172" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R173" r:id="rId514"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId517"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId515"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17864,11 +17854,7 @@
           <t>https://front.alforaij.com/Listing/Detail/295</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/fc7bfde9738d42948d749889a9fd9045.png</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -18296,11 +18282,7 @@
           <t>https://front.alforaij.com/Listing/Detail/279</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/8fd44f6b937742e4b64fccbaf940d5c3.png</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -27170,317 +27152,315 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R84" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R85" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R86" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R87" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R88" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R89" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R90" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R91" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R92" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R93" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R94" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R95" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R96" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q97" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R97" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R98" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R99" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R100" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R101" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q102" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R102" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q103" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R103" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q104" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R104" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q105" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R105" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q106" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R106" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q107" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R107" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q108" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R108" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q109" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R109" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q110" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R110" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q111" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R111" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q112" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R112" r:id="rId331"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId334"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId332"/>
   </tableParts>
 </worksheet>
 </file>
@@ -31331,11 +31311,7 @@
           <t>https://front.alforaij.com/Listing/Detail/279</t>
         </is>
       </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>https://search.alforaij.com/uploads/internallistings/8fd44f6b937742e4b64fccbaf940d5c3.png</t>
-        </is>
-      </c>
+      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -37891,227 +37867,226 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R51" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R52" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R53" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R54" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R55" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R56" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R57" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R62" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R63" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R64" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R65" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R66" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R67" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R75" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R76" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R77" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R78" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R79" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R80" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R81" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R82" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R83" r:id="rId245"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId247"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId246"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>